<commit_message>
templates: add discharge/res-summary/sc + ignore prime/ obsidian vault
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template/ges-prod.xlsx
+++ b/template/ges-prod.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\go\srmt-prime\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\go\srmt-prime\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4968EBA1-E5C3-44B0-8DBC-FFCDF54EAB54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DFE0DF7-8CEF-4459-AC43-5AD4C9E98012}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{580E0F64-EAB3-4BA3-8103-B8D5C69105A5}"/>
   </bookViews>
@@ -610,7 +610,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="18">
+  <numFmts count="21">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0&quot;ºС&quot;"/>
@@ -625,10 +625,13 @@
     <numFmt numFmtId="175" formatCode="#\ ##0.000"/>
     <numFmt numFmtId="176" formatCode="#\ ##0.0000"/>
     <numFmt numFmtId="177" formatCode="0&quot; январь кунги ҳолат прогнози:&quot;"/>
-    <numFmt numFmtId="178" formatCode="0&quot; март кунги ҳолат прогнози:&quot;"/>
     <numFmt numFmtId="179" formatCode="dd/mm/yyyy\ \й\и\л"/>
     <numFmt numFmtId="180" formatCode="yyyy\ \й\и\л"/>
     <numFmt numFmtId="181" formatCode="dd\ mmmm"/>
+    <numFmt numFmtId="182" formatCode="[$-FC19]d\ mmmm\ yyyy\ &quot;г.&quot;"/>
+    <numFmt numFmtId="184" formatCode="mmmm&quot; ойи прогнози:&quot;"/>
+    <numFmt numFmtId="185" formatCode="dd\ mmmm&quot; кунги холат прогнози:&quot;"/>
+    <numFmt numFmtId="186" formatCode="yyyy&quot; йил прогнози:&quot;"/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -1128,13 +1131,7 @@
     <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="177" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1307,6 +1304,63 @@
     <xf numFmtId="0" fontId="21" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="3" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="3" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="9" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="181" fontId="3" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1322,24 +1376,6 @@
     <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="9" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="178" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1349,50 +1385,17 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="3" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="3" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90" wrapText="1"/>
+    <xf numFmtId="182" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="184" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="185" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="186" fontId="9" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1748,215 +1751,215 @@
   <sheetData>
     <row r="1" spans="1:37" ht="12.75" hidden="1" customHeight="1"/>
     <row r="2" spans="1:37" ht="15.75" hidden="1" customHeight="1">
-      <c r="A2" s="129" t="s">
+      <c r="A2" s="113" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="129"/>
-      <c r="C2" s="129"/>
-      <c r="D2" s="129"/>
-      <c r="E2" s="129"/>
-      <c r="F2" s="129"/>
-      <c r="G2" s="129"/>
-      <c r="H2" s="129"/>
-      <c r="I2" s="129"/>
-      <c r="J2" s="129"/>
-      <c r="K2" s="129"/>
-      <c r="L2" s="129"/>
-      <c r="M2" s="129"/>
-      <c r="N2" s="129"/>
-      <c r="O2" s="129"/>
-      <c r="P2" s="129"/>
-      <c r="Q2" s="129"/>
-      <c r="R2" s="129"/>
-      <c r="S2" s="129"/>
-      <c r="T2" s="129"/>
-      <c r="U2" s="129"/>
-      <c r="V2" s="129"/>
-      <c r="W2" s="129"/>
-      <c r="X2" s="129"/>
-      <c r="Y2" s="129"/>
-      <c r="Z2" s="129"/>
-      <c r="AA2" s="129"/>
-      <c r="AB2" s="129"/>
-      <c r="AC2" s="129"/>
-      <c r="AD2" s="129"/>
-      <c r="AE2" s="129"/>
-      <c r="AF2" s="129"/>
-      <c r="AG2" s="129"/>
-      <c r="AH2" s="129"/>
-      <c r="AI2" s="129"/>
-      <c r="AJ2" s="129"/>
-      <c r="AK2" s="129"/>
+      <c r="B2" s="113"/>
+      <c r="C2" s="113"/>
+      <c r="D2" s="113"/>
+      <c r="E2" s="113"/>
+      <c r="F2" s="113"/>
+      <c r="G2" s="113"/>
+      <c r="H2" s="113"/>
+      <c r="I2" s="113"/>
+      <c r="J2" s="113"/>
+      <c r="K2" s="113"/>
+      <c r="L2" s="113"/>
+      <c r="M2" s="113"/>
+      <c r="N2" s="113"/>
+      <c r="O2" s="113"/>
+      <c r="P2" s="113"/>
+      <c r="Q2" s="113"/>
+      <c r="R2" s="113"/>
+      <c r="S2" s="113"/>
+      <c r="T2" s="113"/>
+      <c r="U2" s="113"/>
+      <c r="V2" s="113"/>
+      <c r="W2" s="113"/>
+      <c r="X2" s="113"/>
+      <c r="Y2" s="113"/>
+      <c r="Z2" s="113"/>
+      <c r="AA2" s="113"/>
+      <c r="AB2" s="113"/>
+      <c r="AC2" s="113"/>
+      <c r="AD2" s="113"/>
+      <c r="AE2" s="113"/>
+      <c r="AF2" s="113"/>
+      <c r="AG2" s="113"/>
+      <c r="AH2" s="113"/>
+      <c r="AI2" s="113"/>
+      <c r="AJ2" s="113"/>
+      <c r="AK2" s="113"/>
     </row>
     <row r="3" spans="1:37" ht="52.5" customHeight="1">
-      <c r="A3" s="114" t="s">
+      <c r="A3" s="112" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="111"/>
-      <c r="C3" s="113"/>
-      <c r="D3" s="111"/>
-      <c r="E3" s="110"/>
-      <c r="F3" s="110"/>
-      <c r="G3" s="110"/>
-      <c r="H3" s="110"/>
-      <c r="I3" s="110"/>
-      <c r="J3" s="110"/>
-      <c r="K3" s="110"/>
-      <c r="L3" s="110"/>
-      <c r="M3" s="110"/>
-      <c r="N3" s="110"/>
-      <c r="O3" s="110"/>
-      <c r="P3" s="110"/>
-      <c r="Q3" s="110"/>
-      <c r="R3" s="110"/>
-      <c r="S3" s="112"/>
-      <c r="T3" s="110"/>
-      <c r="U3" s="110"/>
-      <c r="V3" s="110"/>
-      <c r="W3" s="110"/>
-      <c r="X3" s="111"/>
-      <c r="Y3" s="111"/>
-      <c r="Z3" s="111"/>
-      <c r="AA3" s="110"/>
-      <c r="AB3" s="111"/>
-      <c r="AC3" s="111"/>
-      <c r="AD3" s="111"/>
-      <c r="AE3" s="111"/>
-      <c r="AF3" s="111"/>
-      <c r="AG3" s="111"/>
-      <c r="AH3" s="118">
+      <c r="B3" s="109"/>
+      <c r="C3" s="111"/>
+      <c r="D3" s="109"/>
+      <c r="E3" s="108"/>
+      <c r="F3" s="108"/>
+      <c r="G3" s="108"/>
+      <c r="H3" s="108"/>
+      <c r="I3" s="108"/>
+      <c r="J3" s="108"/>
+      <c r="K3" s="108"/>
+      <c r="L3" s="108"/>
+      <c r="M3" s="108"/>
+      <c r="N3" s="108"/>
+      <c r="O3" s="108"/>
+      <c r="P3" s="108"/>
+      <c r="Q3" s="108"/>
+      <c r="R3" s="108"/>
+      <c r="S3" s="110"/>
+      <c r="T3" s="108"/>
+      <c r="U3" s="108"/>
+      <c r="V3" s="108"/>
+      <c r="W3" s="108"/>
+      <c r="X3" s="109"/>
+      <c r="Y3" s="109"/>
+      <c r="Z3" s="109"/>
+      <c r="AA3" s="108"/>
+      <c r="AB3" s="109"/>
+      <c r="AC3" s="109"/>
+      <c r="AD3" s="109"/>
+      <c r="AE3" s="109"/>
+      <c r="AF3" s="109"/>
+      <c r="AG3" s="109"/>
+      <c r="AH3" s="135">
         <v>46094</v>
       </c>
-      <c r="AI3" s="118"/>
-      <c r="AJ3" s="118"/>
-      <c r="AK3" s="118"/>
+      <c r="AI3" s="135"/>
+      <c r="AJ3" s="135"/>
+      <c r="AK3" s="135"/>
     </row>
     <row r="4" spans="1:37" s="10" customFormat="1" ht="33" customHeight="1">
-      <c r="A4" s="130" t="s">
+      <c r="A4" s="114" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="131" t="s">
+      <c r="B4" s="115" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="134">
+      <c r="C4" s="118">
         <f>$AH$3</f>
         <v>46094</v>
       </c>
-      <c r="D4" s="134"/>
-      <c r="E4" s="134"/>
-      <c r="F4" s="134"/>
-      <c r="G4" s="134"/>
-      <c r="H4" s="134"/>
-      <c r="I4" s="134"/>
-      <c r="J4" s="134"/>
-      <c r="K4" s="134"/>
-      <c r="L4" s="134"/>
-      <c r="M4" s="134"/>
-      <c r="N4" s="134"/>
-      <c r="O4" s="134"/>
-      <c r="P4" s="134"/>
-      <c r="Q4" s="134"/>
-      <c r="R4" s="134"/>
-      <c r="S4" s="134"/>
-      <c r="T4" s="134"/>
-      <c r="U4" s="134"/>
-      <c r="V4" s="134"/>
-      <c r="W4" s="134"/>
-      <c r="X4" s="134"/>
-      <c r="Y4" s="135"/>
-      <c r="Z4" s="135">
+      <c r="D4" s="118"/>
+      <c r="E4" s="118"/>
+      <c r="F4" s="118"/>
+      <c r="G4" s="118"/>
+      <c r="H4" s="118"/>
+      <c r="I4" s="118"/>
+      <c r="J4" s="118"/>
+      <c r="K4" s="118"/>
+      <c r="L4" s="118"/>
+      <c r="M4" s="118"/>
+      <c r="N4" s="118"/>
+      <c r="O4" s="118"/>
+      <c r="P4" s="118"/>
+      <c r="Q4" s="118"/>
+      <c r="R4" s="118"/>
+      <c r="S4" s="118"/>
+      <c r="T4" s="118"/>
+      <c r="U4" s="118"/>
+      <c r="V4" s="118"/>
+      <c r="W4" s="118"/>
+      <c r="X4" s="118"/>
+      <c r="Y4" s="119"/>
+      <c r="Z4" s="119">
         <f>DATE(YEAR($AH$3)-1,MONTH($AH$3),DAY($AH$3))</f>
         <v>45729</v>
       </c>
-      <c r="AA4" s="136"/>
-      <c r="AB4" s="136"/>
-      <c r="AC4" s="136"/>
-      <c r="AD4" s="136"/>
-      <c r="AE4" s="136"/>
-      <c r="AF4" s="136"/>
-      <c r="AG4" s="136"/>
-      <c r="AH4" s="136"/>
-      <c r="AI4" s="136"/>
-      <c r="AJ4" s="136"/>
-      <c r="AK4" s="137"/>
+      <c r="AA4" s="120"/>
+      <c r="AB4" s="120"/>
+      <c r="AC4" s="120"/>
+      <c r="AD4" s="120"/>
+      <c r="AE4" s="120"/>
+      <c r="AF4" s="120"/>
+      <c r="AG4" s="120"/>
+      <c r="AH4" s="120"/>
+      <c r="AI4" s="120"/>
+      <c r="AJ4" s="120"/>
+      <c r="AK4" s="121"/>
     </row>
     <row r="5" spans="1:37" s="10" customFormat="1" ht="49.5" customHeight="1">
-      <c r="A5" s="130"/>
-      <c r="B5" s="132"/>
-      <c r="C5" s="141" t="str">
+      <c r="A5" s="114"/>
+      <c r="B5" s="116"/>
+      <c r="C5" s="125" t="str">
         <f>"Режа (Январь-"&amp;PROPER(TEXT($AH$3,"ММММ"))&amp;")"</f>
         <v>Режа (Январь-Март)</v>
       </c>
-      <c r="D5" s="115">
+      <c r="D5" s="132">
         <f>$AH$3 - 1</f>
         <v>46093</v>
       </c>
-      <c r="E5" s="116"/>
-      <c r="F5" s="116"/>
-      <c r="G5" s="116"/>
-      <c r="H5" s="116"/>
-      <c r="I5" s="116"/>
-      <c r="J5" s="116"/>
-      <c r="K5" s="116"/>
-      <c r="L5" s="116"/>
-      <c r="M5" s="116"/>
-      <c r="N5" s="116"/>
-      <c r="O5" s="116"/>
-      <c r="P5" s="116"/>
-      <c r="Q5" s="116"/>
-      <c r="R5" s="116"/>
-      <c r="S5" s="116"/>
-      <c r="T5" s="116"/>
-      <c r="U5" s="117"/>
-      <c r="V5" s="143" t="s">
+      <c r="E5" s="133"/>
+      <c r="F5" s="133"/>
+      <c r="G5" s="133"/>
+      <c r="H5" s="133"/>
+      <c r="I5" s="133"/>
+      <c r="J5" s="133"/>
+      <c r="K5" s="133"/>
+      <c r="L5" s="133"/>
+      <c r="M5" s="133"/>
+      <c r="N5" s="133"/>
+      <c r="O5" s="133"/>
+      <c r="P5" s="133"/>
+      <c r="Q5" s="133"/>
+      <c r="R5" s="133"/>
+      <c r="S5" s="133"/>
+      <c r="T5" s="133"/>
+      <c r="U5" s="134"/>
+      <c r="V5" s="127" t="s">
         <v>35</v>
       </c>
-      <c r="W5" s="143" t="s">
+      <c r="W5" s="127" t="s">
         <v>34</v>
       </c>
-      <c r="X5" s="138" t="s">
+      <c r="X5" s="122" t="s">
         <v>33</v>
       </c>
-      <c r="Y5" s="139"/>
-      <c r="Z5" s="115">
+      <c r="Y5" s="123"/>
+      <c r="Z5" s="132">
         <f>$AH$3 - 1</f>
         <v>46093</v>
       </c>
-      <c r="AA5" s="116"/>
-      <c r="AB5" s="116"/>
-      <c r="AC5" s="116"/>
-      <c r="AD5" s="116"/>
-      <c r="AE5" s="116"/>
-      <c r="AF5" s="116"/>
-      <c r="AG5" s="116"/>
-      <c r="AH5" s="126" t="s">
+      <c r="AA5" s="133"/>
+      <c r="AB5" s="133"/>
+      <c r="AC5" s="133"/>
+      <c r="AD5" s="133"/>
+      <c r="AE5" s="133"/>
+      <c r="AF5" s="133"/>
+      <c r="AG5" s="133"/>
+      <c r="AH5" s="137" t="s">
         <v>32</v>
       </c>
-      <c r="AI5" s="128" t="s">
+      <c r="AI5" s="139" t="s">
         <v>31</v>
       </c>
-      <c r="AJ5" s="140" t="s">
+      <c r="AJ5" s="124" t="s">
         <v>30</v>
       </c>
-      <c r="AK5" s="140"/>
+      <c r="AK5" s="124"/>
     </row>
     <row r="6" spans="1:37" s="10" customFormat="1" ht="369.9" customHeight="1">
-      <c r="A6" s="130"/>
-      <c r="B6" s="133"/>
-      <c r="C6" s="142"/>
+      <c r="A6" s="114"/>
+      <c r="B6" s="117"/>
+      <c r="C6" s="126"/>
       <c r="D6" s="16" t="s">
         <v>13</v>
       </c>
       <c r="E6" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="109" t="s">
+      <c r="F6" s="107" t="s">
         <v>29</v>
       </c>
       <c r="G6" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="H6" s="109" t="s">
+      <c r="H6" s="107" t="s">
         <v>27</v>
       </c>
       <c r="I6" s="16" t="s">
@@ -1998,8 +2001,8 @@
       <c r="U6" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="V6" s="143"/>
-      <c r="W6" s="143"/>
+      <c r="V6" s="127"/>
+      <c r="W6" s="127"/>
       <c r="X6" s="15" t="s">
         <v>15</v>
       </c>
@@ -2030,8 +2033,8 @@
       <c r="AG6" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="AH6" s="127"/>
-      <c r="AI6" s="127"/>
+      <c r="AH6" s="138"/>
+      <c r="AI6" s="138"/>
       <c r="AJ6" s="18" t="s">
         <v>5</v>
       </c>
@@ -2040,175 +2043,175 @@
       </c>
     </row>
     <row r="7" spans="1:37" s="11" customFormat="1" ht="54" customHeight="1">
-      <c r="A7" s="78"/>
-      <c r="B7" s="97"/>
-      <c r="C7" s="89"/>
-      <c r="D7" s="100"/>
-      <c r="E7" s="92"/>
-      <c r="F7" s="92"/>
-      <c r="G7" s="98"/>
-      <c r="H7" s="98"/>
-      <c r="I7" s="99"/>
-      <c r="J7" s="98"/>
-      <c r="K7" s="98"/>
-      <c r="L7" s="98"/>
-      <c r="M7" s="98"/>
-      <c r="N7" s="98"/>
-      <c r="O7" s="91"/>
-      <c r="P7" s="97"/>
-      <c r="Q7" s="97"/>
-      <c r="R7" s="87"/>
-      <c r="S7" s="96"/>
-      <c r="T7" s="73"/>
-      <c r="U7" s="95"/>
-      <c r="V7" s="91"/>
-      <c r="W7" s="90"/>
-      <c r="X7" s="94"/>
-      <c r="Y7" s="87"/>
-      <c r="Z7" s="93"/>
-      <c r="AA7" s="92"/>
-      <c r="AB7" s="87"/>
-      <c r="AC7" s="87"/>
-      <c r="AD7" s="87"/>
-      <c r="AE7" s="87"/>
-      <c r="AF7" s="89"/>
-      <c r="AG7" s="91"/>
-      <c r="AH7" s="90"/>
-      <c r="AI7" s="89"/>
-      <c r="AJ7" s="88"/>
-      <c r="AK7" s="87"/>
+      <c r="A7" s="76"/>
+      <c r="B7" s="95"/>
+      <c r="C7" s="87"/>
+      <c r="D7" s="98"/>
+      <c r="E7" s="90"/>
+      <c r="F7" s="90"/>
+      <c r="G7" s="96"/>
+      <c r="H7" s="96"/>
+      <c r="I7" s="97"/>
+      <c r="J7" s="96"/>
+      <c r="K7" s="96"/>
+      <c r="L7" s="96"/>
+      <c r="M7" s="96"/>
+      <c r="N7" s="96"/>
+      <c r="O7" s="89"/>
+      <c r="P7" s="95"/>
+      <c r="Q7" s="95"/>
+      <c r="R7" s="85"/>
+      <c r="S7" s="94"/>
+      <c r="T7" s="71"/>
+      <c r="U7" s="93"/>
+      <c r="V7" s="89"/>
+      <c r="W7" s="88"/>
+      <c r="X7" s="92"/>
+      <c r="Y7" s="85"/>
+      <c r="Z7" s="91"/>
+      <c r="AA7" s="90"/>
+      <c r="AB7" s="85"/>
+      <c r="AC7" s="85"/>
+      <c r="AD7" s="85"/>
+      <c r="AE7" s="85"/>
+      <c r="AF7" s="87"/>
+      <c r="AG7" s="89"/>
+      <c r="AH7" s="88"/>
+      <c r="AI7" s="87"/>
+      <c r="AJ7" s="86"/>
+      <c r="AK7" s="85"/>
     </row>
     <row r="8" spans="1:37" s="14" customFormat="1" ht="30.75" customHeight="1">
-      <c r="A8" s="106"/>
-      <c r="B8" s="81"/>
-      <c r="C8" s="107"/>
-      <c r="D8" s="85"/>
-      <c r="E8" s="79"/>
-      <c r="F8" s="86"/>
-      <c r="G8" s="81"/>
-      <c r="H8" s="84"/>
-      <c r="I8" s="101"/>
-      <c r="J8" s="103"/>
-      <c r="K8" s="84"/>
-      <c r="L8" s="103"/>
-      <c r="M8" s="103"/>
-      <c r="N8" s="84"/>
-      <c r="O8" s="82"/>
-      <c r="P8" s="105"/>
-      <c r="Q8" s="105"/>
-      <c r="R8" s="81"/>
-      <c r="S8" s="84"/>
-      <c r="T8" s="102"/>
-      <c r="U8" s="83"/>
-      <c r="V8" s="79"/>
-      <c r="W8" s="79"/>
-      <c r="X8" s="104"/>
-      <c r="Y8" s="107"/>
-      <c r="Z8" s="85"/>
-      <c r="AA8" s="80"/>
-      <c r="AB8" s="81"/>
-      <c r="AC8" s="81"/>
-      <c r="AD8" s="103"/>
-      <c r="AE8" s="103"/>
-      <c r="AF8" s="81"/>
-      <c r="AG8" s="79"/>
-      <c r="AH8" s="79"/>
-      <c r="AI8" s="81"/>
-      <c r="AJ8" s="108"/>
-      <c r="AK8" s="108"/>
+      <c r="A8" s="104"/>
+      <c r="B8" s="79"/>
+      <c r="C8" s="105"/>
+      <c r="D8" s="83"/>
+      <c r="E8" s="77"/>
+      <c r="F8" s="84"/>
+      <c r="G8" s="79"/>
+      <c r="H8" s="82"/>
+      <c r="I8" s="99"/>
+      <c r="J8" s="101"/>
+      <c r="K8" s="82"/>
+      <c r="L8" s="101"/>
+      <c r="M8" s="101"/>
+      <c r="N8" s="82"/>
+      <c r="O8" s="80"/>
+      <c r="P8" s="103"/>
+      <c r="Q8" s="103"/>
+      <c r="R8" s="79"/>
+      <c r="S8" s="82"/>
+      <c r="T8" s="100"/>
+      <c r="U8" s="81"/>
+      <c r="V8" s="77"/>
+      <c r="W8" s="77"/>
+      <c r="X8" s="102"/>
+      <c r="Y8" s="105"/>
+      <c r="Z8" s="83"/>
+      <c r="AA8" s="78"/>
+      <c r="AB8" s="79"/>
+      <c r="AC8" s="79"/>
+      <c r="AD8" s="101"/>
+      <c r="AE8" s="101"/>
+      <c r="AF8" s="79"/>
+      <c r="AG8" s="77"/>
+      <c r="AH8" s="77"/>
+      <c r="AI8" s="79"/>
+      <c r="AJ8" s="106"/>
+      <c r="AK8" s="106"/>
     </row>
     <row r="9" spans="1:37" s="11" customFormat="1" ht="54" customHeight="1">
-      <c r="A9" s="78" t="s">
+      <c r="A9" s="76" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="70"/>
-      <c r="C9" s="64"/>
-      <c r="D9" s="77"/>
-      <c r="E9" s="69"/>
-      <c r="F9" s="69"/>
-      <c r="G9" s="75"/>
-      <c r="H9" s="75"/>
-      <c r="I9" s="76"/>
-      <c r="J9" s="75"/>
-      <c r="K9" s="75"/>
-      <c r="L9" s="75"/>
-      <c r="M9" s="75"/>
-      <c r="N9" s="75"/>
-      <c r="O9" s="67"/>
-      <c r="P9" s="70"/>
-      <c r="Q9" s="70"/>
-      <c r="R9" s="64"/>
-      <c r="S9" s="74"/>
-      <c r="T9" s="73"/>
-      <c r="U9" s="72"/>
-      <c r="V9" s="67"/>
-      <c r="W9" s="67"/>
-      <c r="X9" s="71"/>
-      <c r="Y9" s="70"/>
-      <c r="Z9" s="69"/>
-      <c r="AA9" s="69"/>
-      <c r="AB9" s="64"/>
-      <c r="AC9" s="64"/>
-      <c r="AD9" s="64"/>
-      <c r="AE9" s="64"/>
-      <c r="AF9" s="68"/>
-      <c r="AG9" s="67"/>
-      <c r="AH9" s="66"/>
-      <c r="AI9" s="66"/>
-      <c r="AJ9" s="65"/>
-      <c r="AK9" s="64"/>
+      <c r="B9" s="68"/>
+      <c r="C9" s="62"/>
+      <c r="D9" s="75"/>
+      <c r="E9" s="67"/>
+      <c r="F9" s="67"/>
+      <c r="G9" s="73"/>
+      <c r="H9" s="73"/>
+      <c r="I9" s="74"/>
+      <c r="J9" s="73"/>
+      <c r="K9" s="73"/>
+      <c r="L9" s="73"/>
+      <c r="M9" s="73"/>
+      <c r="N9" s="73"/>
+      <c r="O9" s="65"/>
+      <c r="P9" s="68"/>
+      <c r="Q9" s="68"/>
+      <c r="R9" s="62"/>
+      <c r="S9" s="72"/>
+      <c r="T9" s="71"/>
+      <c r="U9" s="70"/>
+      <c r="V9" s="65"/>
+      <c r="W9" s="65"/>
+      <c r="X9" s="69"/>
+      <c r="Y9" s="68"/>
+      <c r="Z9" s="67"/>
+      <c r="AA9" s="67"/>
+      <c r="AB9" s="62"/>
+      <c r="AC9" s="62"/>
+      <c r="AD9" s="62"/>
+      <c r="AE9" s="62"/>
+      <c r="AF9" s="66"/>
+      <c r="AG9" s="65"/>
+      <c r="AH9" s="64"/>
+      <c r="AI9" s="64"/>
+      <c r="AJ9" s="63"/>
+      <c r="AK9" s="62"/>
     </row>
     <row r="10" spans="1:37" ht="37.5" customHeight="1">
       <c r="A10" s="17"/>
       <c r="B10" s="20"/>
-      <c r="C10" s="63"/>
-      <c r="D10" s="59"/>
-      <c r="E10" s="59"/>
-      <c r="F10" s="59"/>
-      <c r="G10" s="59"/>
-      <c r="H10" s="59"/>
-      <c r="I10" s="59"/>
-      <c r="J10" s="59"/>
-      <c r="K10" s="59"/>
-      <c r="L10" s="61"/>
-      <c r="M10" s="61"/>
-      <c r="N10" s="61"/>
-      <c r="O10" s="123" t="str">
-        <f>YEAR($AH$3)&amp;" йил прогнози:"</f>
-        <v>2026 йил прогнози:</v>
-      </c>
-      <c r="P10" s="123"/>
-      <c r="Q10" s="123"/>
-      <c r="R10" s="123"/>
-      <c r="S10" s="123"/>
-      <c r="T10" s="62">
+      <c r="C10" s="61"/>
+      <c r="D10" s="57"/>
+      <c r="E10" s="57"/>
+      <c r="F10" s="57"/>
+      <c r="G10" s="57"/>
+      <c r="H10" s="57"/>
+      <c r="I10" s="57"/>
+      <c r="J10" s="57"/>
+      <c r="K10" s="57"/>
+      <c r="L10" s="59"/>
+      <c r="M10" s="59"/>
+      <c r="N10" s="59"/>
+      <c r="O10" s="143">
+        <f>$AH$3</f>
+        <v>46094</v>
+      </c>
+      <c r="P10" s="143"/>
+      <c r="Q10" s="143"/>
+      <c r="R10" s="143"/>
+      <c r="S10" s="143"/>
+      <c r="T10" s="60">
         <v>0</v>
       </c>
       <c r="U10" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="V10" s="61"/>
+      <c r="V10" s="59"/>
       <c r="W10" s="47"/>
       <c r="X10" s="20"/>
       <c r="Y10" s="20"/>
-      <c r="Z10" s="60"/>
-      <c r="AA10" s="59"/>
-      <c r="AB10" s="58"/>
-      <c r="AC10" s="58"/>
+      <c r="Z10" s="58"/>
+      <c r="AA10" s="57"/>
+      <c r="AB10" s="56"/>
+      <c r="AC10" s="56"/>
       <c r="AD10" s="20"/>
       <c r="AE10" s="20"/>
-      <c r="AF10" s="55"/>
-      <c r="AG10" s="55"/>
-      <c r="AH10" s="55"/>
-      <c r="AI10" s="55"/>
-      <c r="AJ10" s="55"/>
+      <c r="AF10" s="54"/>
+      <c r="AG10" s="54"/>
+      <c r="AH10" s="54"/>
+      <c r="AI10" s="54"/>
+      <c r="AJ10" s="54"/>
       <c r="AK10" s="20"/>
     </row>
     <row r="11" spans="1:37" ht="30" customHeight="1">
       <c r="A11" s="17"/>
       <c r="B11" s="20"/>
       <c r="C11" s="49"/>
-      <c r="D11" s="57"/>
+      <c r="D11" s="55"/>
       <c r="E11" s="53"/>
       <c r="F11" s="53"/>
       <c r="G11" s="40"/>
@@ -2216,17 +2219,17 @@
       <c r="I11" s="40"/>
       <c r="J11" s="53"/>
       <c r="K11" s="40"/>
-      <c r="L11" s="124" t="str">
-        <f>PROPER(TEXT($AH$3,"ММММ"))&amp;" ойи прогнози:"</f>
-        <v>Март ойи прогнози:</v>
-      </c>
-      <c r="M11" s="124"/>
-      <c r="N11" s="124"/>
-      <c r="O11" s="124"/>
-      <c r="P11" s="124"/>
-      <c r="Q11" s="124"/>
-      <c r="R11" s="124"/>
-      <c r="S11" s="124"/>
+      <c r="L11" s="141">
+        <f>$AH$3</f>
+        <v>46094</v>
+      </c>
+      <c r="M11" s="141"/>
+      <c r="N11" s="141"/>
+      <c r="O11" s="141"/>
+      <c r="P11" s="141"/>
+      <c r="Q11" s="141"/>
+      <c r="R11" s="141"/>
+      <c r="S11" s="141"/>
       <c r="T11" s="13">
         <v>0</v>
       </c>
@@ -2234,14 +2237,14 @@
         <v>2</v>
       </c>
       <c r="V11" s="43"/>
-      <c r="W11" s="56"/>
-      <c r="X11" s="20"/>
-      <c r="Y11" s="55"/>
-      <c r="Z11" s="54"/>
-      <c r="AA11" s="53"/>
-      <c r="AB11" s="51"/>
-      <c r="AC11" s="39"/>
-      <c r="AD11" s="20"/>
+      <c r="W11" s="140"/>
+      <c r="X11" s="140"/>
+      <c r="Y11" s="140"/>
+      <c r="Z11" s="140"/>
+      <c r="AA11" s="140"/>
+      <c r="AB11" s="140"/>
+      <c r="AC11" s="140"/>
+      <c r="AD11" s="140"/>
       <c r="AE11" s="20"/>
       <c r="AF11" s="20"/>
       <c r="AG11" s="20"/>
@@ -2262,17 +2265,17 @@
       <c r="I12" s="40"/>
       <c r="J12" s="40"/>
       <c r="K12" s="40"/>
-      <c r="L12" s="125" t="str">
-        <f>DAY($AH$3)&amp;" "&amp;TEXT($AH$3,"ММММ")&amp;" кунги холат прогнози:"</f>
-        <v>13 Март кунги холат прогнози:</v>
-      </c>
-      <c r="M12" s="125"/>
-      <c r="N12" s="125"/>
-      <c r="O12" s="125"/>
-      <c r="P12" s="125"/>
-      <c r="Q12" s="125"/>
-      <c r="R12" s="125"/>
-      <c r="S12" s="125"/>
+      <c r="L12" s="142">
+        <f>$AH$3</f>
+        <v>46094</v>
+      </c>
+      <c r="M12" s="142"/>
+      <c r="N12" s="142"/>
+      <c r="O12" s="142"/>
+      <c r="P12" s="142"/>
+      <c r="Q12" s="142"/>
+      <c r="R12" s="142"/>
+      <c r="S12" s="142"/>
       <c r="T12" s="13">
         <v>0</v>
       </c>
@@ -2308,16 +2311,16 @@
       <c r="I13" s="40"/>
       <c r="J13" s="40"/>
       <c r="K13" s="40"/>
-      <c r="L13" s="124" t="s">
+      <c r="L13" s="130" t="s">
         <v>3</v>
       </c>
-      <c r="M13" s="124"/>
-      <c r="N13" s="124"/>
-      <c r="O13" s="124"/>
-      <c r="P13" s="124"/>
-      <c r="Q13" s="124"/>
-      <c r="R13" s="124"/>
-      <c r="S13" s="124"/>
+      <c r="M13" s="130"/>
+      <c r="N13" s="130"/>
+      <c r="O13" s="130"/>
+      <c r="P13" s="130"/>
+      <c r="Q13" s="130"/>
+      <c r="R13" s="130"/>
+      <c r="S13" s="130"/>
       <c r="T13" s="13">
         <f>+V9</f>
         <v>0</v>
@@ -2343,33 +2346,33 @@
       <c r="AK13" s="20"/>
     </row>
     <row r="14" spans="1:37" ht="30" customHeight="1">
-      <c r="A14" s="120" t="s">
+      <c r="A14" s="131" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="120"/>
-      <c r="C14" s="120"/>
+      <c r="B14" s="131"/>
+      <c r="C14" s="131"/>
       <c r="D14" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="E14" s="121">
+      <c r="E14" s="129">
         <v>0</v>
       </c>
-      <c r="F14" s="121"/>
+      <c r="F14" s="129"/>
       <c r="G14" s="40"/>
       <c r="H14" s="40"/>
       <c r="I14" s="40"/>
       <c r="J14" s="40"/>
       <c r="K14" s="40"/>
-      <c r="L14" s="124" t="s">
+      <c r="L14" s="130" t="s">
         <v>1</v>
       </c>
-      <c r="M14" s="124"/>
-      <c r="N14" s="124"/>
-      <c r="O14" s="124"/>
-      <c r="P14" s="124"/>
-      <c r="Q14" s="124"/>
-      <c r="R14" s="124"/>
-      <c r="S14" s="124"/>
+      <c r="M14" s="130"/>
+      <c r="N14" s="130"/>
+      <c r="O14" s="130"/>
+      <c r="P14" s="130"/>
+      <c r="Q14" s="130"/>
+      <c r="R14" s="130"/>
+      <c r="S14" s="130"/>
       <c r="T14" s="13">
         <f>IFERROR(T13/T11*100,0)</f>
         <v>0</v>
@@ -2395,19 +2398,19 @@
       <c r="AK14" s="20"/>
     </row>
     <row r="15" spans="1:37" ht="30" customHeight="1">
-      <c r="A15" s="120" t="s">
+      <c r="A15" s="131" t="s">
         <v>44</v>
       </c>
-      <c r="B15" s="120"/>
-      <c r="C15" s="120"/>
+      <c r="B15" s="131"/>
+      <c r="C15" s="131"/>
       <c r="D15" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="E15" s="121">
+      <c r="E15" s="129">
         <f>+P9</f>
         <v>0</v>
       </c>
-      <c r="F15" s="121"/>
+      <c r="F15" s="129"/>
       <c r="G15" s="30" t="s">
         <v>43</v>
       </c>
@@ -2445,19 +2448,19 @@
       <c r="AK15" s="26"/>
     </row>
     <row r="16" spans="1:37" ht="30" customHeight="1">
-      <c r="A16" s="122" t="s">
+      <c r="A16" s="128" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="122"/>
-      <c r="C16" s="122"/>
+      <c r="B16" s="128"/>
+      <c r="C16" s="128"/>
       <c r="D16" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="E16" s="121">
+      <c r="E16" s="129">
         <f>+Q9</f>
         <v>0</v>
       </c>
-      <c r="F16" s="121"/>
+      <c r="F16" s="129"/>
       <c r="G16" s="30"/>
       <c r="H16" s="30"/>
       <c r="I16" s="30"/>
@@ -2491,19 +2494,19 @@
       <c r="AK16" s="26"/>
     </row>
     <row r="17" spans="1:37" ht="30" customHeight="1">
-      <c r="A17" s="122" t="s">
+      <c r="A17" s="128" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="122"/>
-      <c r="C17" s="122"/>
+      <c r="B17" s="128"/>
+      <c r="C17" s="128"/>
       <c r="D17" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="E17" s="121">
+      <c r="E17" s="129">
         <f>+E15-E16-E18-E19</f>
         <v>-18</v>
       </c>
-      <c r="F17" s="121"/>
+      <c r="F17" s="129"/>
       <c r="G17" s="30"/>
       <c r="H17" s="30"/>
       <c r="I17" s="30"/>
@@ -2539,18 +2542,18 @@
       <c r="AK17" s="26"/>
     </row>
     <row r="18" spans="1:37" ht="30" customHeight="1">
-      <c r="A18" s="122" t="s">
+      <c r="A18" s="128" t="s">
         <v>40</v>
       </c>
-      <c r="B18" s="122"/>
-      <c r="C18" s="122"/>
+      <c r="B18" s="128"/>
+      <c r="C18" s="128"/>
       <c r="D18" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="E18" s="121">
+      <c r="E18" s="129">
         <v>14</v>
       </c>
-      <c r="F18" s="121"/>
+      <c r="F18" s="129"/>
       <c r="G18" s="26"/>
       <c r="H18" s="26"/>
       <c r="I18" s="26"/>
@@ -2584,24 +2587,24 @@
       <c r="AK18" s="26"/>
     </row>
     <row r="19" spans="1:37" ht="30" customHeight="1">
-      <c r="A19" s="122" t="s">
+      <c r="A19" s="128" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="122"/>
-      <c r="C19" s="122"/>
+      <c r="B19" s="128"/>
+      <c r="C19" s="128"/>
       <c r="D19" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="E19" s="121">
+      <c r="E19" s="129">
         <v>4</v>
       </c>
-      <c r="F19" s="121"/>
+      <c r="F19" s="129"/>
       <c r="G19" s="22"/>
       <c r="H19" s="22"/>
-      <c r="I19" s="119"/>
-      <c r="J19" s="119"/>
-      <c r="K19" s="119"/>
-      <c r="L19" s="119"/>
+      <c r="I19" s="136"/>
+      <c r="J19" s="136"/>
+      <c r="K19" s="136"/>
+      <c r="L19" s="136"/>
       <c r="M19" s="22"/>
       <c r="N19" s="22"/>
       <c r="O19" s="22"/>
@@ -2611,9 +2614,9 @@
       <c r="S19" s="22"/>
       <c r="T19" s="22"/>
       <c r="U19" s="22"/>
-      <c r="V19" s="119"/>
-      <c r="W19" s="119"/>
-      <c r="X19" s="119"/>
+      <c r="V19" s="136"/>
+      <c r="W19" s="136"/>
+      <c r="X19" s="136"/>
       <c r="Y19" s="21"/>
       <c r="Z19" s="23"/>
       <c r="AA19" s="22"/>
@@ -3097,17 +3100,16 @@
       <c r="AK31" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="34">
-    <mergeCell ref="A2:AK2"/>
-    <mergeCell ref="A4:A6"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="C4:Y4"/>
-    <mergeCell ref="Z4:AK4"/>
-    <mergeCell ref="X5:Y5"/>
-    <mergeCell ref="AJ5:AK5"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="V5:V6"/>
-    <mergeCell ref="W5:W6"/>
+  <mergeCells count="35">
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="D5:U5"/>
+    <mergeCell ref="Z5:AG5"/>
+    <mergeCell ref="AH3:AK3"/>
+    <mergeCell ref="I19:L19"/>
+    <mergeCell ref="V19:X19"/>
+    <mergeCell ref="AH5:AH6"/>
+    <mergeCell ref="AI5:AI6"/>
+    <mergeCell ref="W11:AD11"/>
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="E18:F18"/>
     <mergeCell ref="A19:C19"/>
@@ -3124,14 +3126,16 @@
     <mergeCell ref="A16:C16"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="A17:C17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="D5:U5"/>
-    <mergeCell ref="Z5:AG5"/>
-    <mergeCell ref="AH3:AK3"/>
-    <mergeCell ref="I19:L19"/>
-    <mergeCell ref="V19:X19"/>
-    <mergeCell ref="AH5:AH6"/>
-    <mergeCell ref="AI5:AI6"/>
+    <mergeCell ref="A2:AK2"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="C4:Y4"/>
+    <mergeCell ref="Z4:AK4"/>
+    <mergeCell ref="X5:Y5"/>
+    <mergeCell ref="AJ5:AK5"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="V5:V6"/>
+    <mergeCell ref="W5:W6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="7.8740157480315001E-2" right="7.8740157480315001E-2" top="0.39370078740157499" bottom="7.8740157480315001E-2" header="0.43307086614173201" footer="0.31496062992126"/>

</xml_diff>